<commit_message>
feat(productos): guion de la Guía Food Cost (20 caps + 12 ejercicios, 461 referencias a celda verificadas, 0 rotas) · documentos.py toma versión y fecha del guion · Goal Value como índice sin € en la matriz
Via: Claude Code

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KT5bueRhJ8E1oD5EU8zzPS
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/guia-food-cost-ingenieria-menu/matriz-multimetodo-carta.xlsx
+++ b/astro-site/public/dl/guia-food-cost-ingenieria-menu/matriz-multimetodo-carta.xlsx
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +139,8 @@
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -7679,7 +7681,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>Distancia al objetivo (€)</t>
+          <t>Distancia al objetivo (índice)</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr">
@@ -7712,7 +7714,7 @@
         <f>IFERROR(IF('Datos'!$F5="","",'Datos'!$F5),"")</f>
         <v>8.6</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="22">
         <f>IFERROR(IF(OR($D5="",$E5="",$F5="",$D$33+$D$34+$E5&gt;=1),"",(1-$E5)*$D5*$F5*(1-($D$33+$D$34+$E5))),"")</f>
         <v>916.7720930232557</v>
       </c>
@@ -7728,7 +7730,7 @@
         <f>IFERROR(IF('Datos'!$O5="","",'Datos'!$O5),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K5" s="13">
+      <c r="K5" s="23">
         <f>IFERROR(IF(OR($H5="",$I5="",$J5="",$D$33+$D$34+$J5&gt;=1),"",(1-$J5)*$H5*$I5*(1-($D$33+$D$34+$J5))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -7736,7 +7738,7 @@
         <f>IFERROR(IF(OR($G5="",$K5=""),"",IF($G5&gt;=$K5,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M5" s="13">
+      <c r="M5" s="23">
         <f>IFERROR(IF(OR($G5="",$K5=""),"",$G5-$K5),"")</f>
         <v>413.47608713603285</v>
       </c>
@@ -7769,7 +7771,7 @@
         <f>IFERROR(IF('Datos'!$F6="","",'Datos'!$F6),"")</f>
         <v>11.8</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="22">
         <f>IFERROR(IF(OR($D6="",$E6="",$F6="",$D$33+$D$34+$E6&gt;=1),"",(1-$E6)*$D6*$F6*(1-($D$33+$D$34+$E6))),"")</f>
         <v>698.8345762711865</v>
       </c>
@@ -7785,7 +7787,7 @@
         <f>IFERROR(IF('Datos'!$O6="","",'Datos'!$O6),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="23">
         <f>IFERROR(IF(OR($H6="",$I6="",$J6="",$D$33+$D$34+$J6&gt;=1),"",(1-$J6)*$H6*$I6*(1-($D$33+$D$34+$J6))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -7793,7 +7795,7 @@
         <f>IFERROR(IF(OR($G6="",$K6=""),"",IF($G6&gt;=$K6,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M6" s="13">
+      <c r="M6" s="23">
         <f>IFERROR(IF(OR($G6="",$K6=""),"",$G6-$K6),"")</f>
         <v>195.53857038396364</v>
       </c>
@@ -7826,7 +7828,7 @@
         <f>IFERROR(IF('Datos'!$F7="","",'Datos'!$F7),"")</f>
         <v>15.5</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="22">
         <f>IFERROR(IF(OR($D7="",$E7="",$F7="",$D$33+$D$34+$E7&gt;=1),"",(1-$E7)*$D7*$F7*(1-($D$33+$D$34+$E7))),"")</f>
         <v>301.4993548387095</v>
       </c>
@@ -7842,7 +7844,7 @@
         <f>IFERROR(IF('Datos'!$O7="","",'Datos'!$O7),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="23">
         <f>IFERROR(IF(OR($H7="",$I7="",$J7="",$D$33+$D$34+$J7&gt;=1),"",(1-$J7)*$H7*$I7*(1-($D$33+$D$34+$J7))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -7850,7 +7852,7 @@
         <f>IFERROR(IF(OR($G7="",$K7=""),"",IF($G7&gt;=$K7,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M7" s="13">
+      <c r="M7" s="23">
         <f>IFERROR(IF(OR($G7="",$K7=""),"",$G7-$K7),"")</f>
         <v>-201.79665104851335</v>
       </c>
@@ -7883,7 +7885,7 @@
         <f>IFERROR(IF('Datos'!$F8="","",'Datos'!$F8),"")</f>
         <v>9.8</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="22">
         <f>IFERROR(IF(OR($D8="",$E8="",$F8="",$D$33+$D$34+$E8&gt;=1),"",(1-$E8)*$D8*$F8*(1-($D$33+$D$34+$E8))),"")</f>
         <v>942.3069387755104</v>
       </c>
@@ -7899,7 +7901,7 @@
         <f>IFERROR(IF('Datos'!$O8="","",'Datos'!$O8),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="23">
         <f>IFERROR(IF(OR($H8="",$I8="",$J8="",$D$33+$D$34+$J8&gt;=1),"",(1-$J8)*$H8*$I8*(1-($D$33+$D$34+$J8))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -7907,7 +7909,7 @@
         <f>IFERROR(IF(OR($G8="",$K8=""),"",IF($G8&gt;=$K8,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M8" s="13">
+      <c r="M8" s="23">
         <f>IFERROR(IF(OR($G8="",$K8=""),"",$G8-$K8),"")</f>
         <v>439.0109328882875</v>
       </c>
@@ -7940,7 +7942,7 @@
         <f>IFERROR(IF('Datos'!$F9="","",'Datos'!$F9),"")</f>
         <v>13.6</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="22">
         <f>IFERROR(IF(OR($D9="",$E9="",$F9="",$D$33+$D$34+$E9&gt;=1),"",(1-$E9)*$D9*$F9*(1-($D$33+$D$34+$E9))),"")</f>
         <v>149.42117647058814</v>
       </c>
@@ -7956,7 +7958,7 @@
         <f>IFERROR(IF('Datos'!$O9="","",'Datos'!$O9),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K9" s="13">
+      <c r="K9" s="23">
         <f>IFERROR(IF(OR($H9="",$I9="",$J9="",$D$33+$D$34+$J9&gt;=1),"",(1-$J9)*$H9*$I9*(1-($D$33+$D$34+$J9))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -7964,7 +7966,7 @@
         <f>IFERROR(IF(OR($G9="",$K9=""),"",IF($G9&gt;=$K9,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M9" s="13">
+      <c r="M9" s="23">
         <f>IFERROR(IF(OR($G9="",$K9=""),"",$G9-$K9),"")</f>
         <v>-353.8748294166347</v>
       </c>
@@ -7997,7 +7999,7 @@
         <f>IFERROR(IF('Datos'!$F10="","",'Datos'!$F10),"")</f>
         <v>10.9</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="22">
         <f>IFERROR(IF(OR($D10="",$E10="",$F10="",$D$33+$D$34+$E10&gt;=1),"",(1-$E10)*$D10*$F10*(1-($D$33+$D$34+$E10))),"")</f>
         <v>276.67816513761466</v>
       </c>
@@ -8013,7 +8015,7 @@
         <f>IFERROR(IF('Datos'!$O10="","",'Datos'!$O10),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="23">
         <f>IFERROR(IF(OR($H10="",$I10="",$J10="",$D$33+$D$34+$J10&gt;=1),"",(1-$J10)*$H10*$I10*(1-($D$33+$D$34+$J10))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -8021,7 +8023,7 @@
         <f>IFERROR(IF(OR($G10="",$K10=""),"",IF($G10&gt;=$K10,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M10" s="13">
+      <c r="M10" s="23">
         <f>IFERROR(IF(OR($G10="",$K10=""),"",$G10-$K10),"")</f>
         <v>-226.6178407496082</v>
       </c>
@@ -8054,7 +8056,7 @@
         <f>IFERROR(IF('Datos'!$F11="","",'Datos'!$F11),"")</f>
         <v>7.2</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="22">
         <f>IFERROR(IF(OR($D11="",$E11="",$F11="",$D$33+$D$34+$E11&gt;=1),"",(1-$E11)*$D11*$F11*(1-($D$33+$D$34+$E11))),"")</f>
         <v>372.0</v>
       </c>
@@ -8070,7 +8072,7 @@
         <f>IFERROR(IF('Datos'!$O11="","",'Datos'!$O11),"")</f>
         <v>0.3071474565357373</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="23">
         <f>IFERROR(IF(OR($H11="",$I11="",$J11="",$D$33+$D$34+$J11&gt;=1),"",(1-$J11)*$H11*$I11*(1-($D$33+$D$34+$J11))),"")</f>
         <v>503.29600588722286</v>
       </c>
@@ -8078,7 +8080,7 @@
         <f>IFERROR(IF(OR($G11="",$K11=""),"",IF($G11&gt;=$K11,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M11" s="13">
+      <c r="M11" s="23">
         <f>IFERROR(IF(OR($G11="",$K11=""),"",$G11-$K11),"")</f>
         <v>-131.29600588722286</v>
       </c>
@@ -8111,7 +8113,7 @@
         <f>IFERROR(IF('Datos'!$F12="","",'Datos'!$F12),"")</f>
         <v>17.3</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="22">
         <f>IFERROR(IF(OR($D12="",$E12="",$F12="",$D$33+$D$34+$E12&gt;=1),"",(1-$E12)*$D12*$F12*(1-($D$33+$D$34+$E12))),"")</f>
         <v>997.4640924855493</v>
       </c>
@@ -8127,7 +8129,7 @@
         <f>IFERROR(IF('Datos'!$O12="","",'Datos'!$O12),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K12" s="13">
+      <c r="K12" s="23">
         <f>IFERROR(IF(OR($H12="",$I12="",$J12="",$D$33+$D$34+$J12&gt;=1),"",(1-$J12)*$H12*$I12*(1-($D$33+$D$34+$J12))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8135,7 +8137,7 @@
         <f>IFERROR(IF(OR($G12="",$K12=""),"",IF($G12&gt;=$K12,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M12" s="13">
+      <c r="M12" s="23">
         <f>IFERROR(IF(OR($G12="",$K12=""),"",$G12-$K12),"")</f>
         <v>454.42969437076874</v>
       </c>
@@ -8168,7 +8170,7 @@
         <f>IFERROR(IF('Datos'!$F13="","",'Datos'!$F13),"")</f>
         <v>19.1</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="22">
         <f>IFERROR(IF(OR($D13="",$E13="",$F13="",$D$33+$D$34+$E13&gt;=1),"",(1-$E13)*$D13*$F13*(1-($D$33+$D$34+$E13))),"")</f>
         <v>428.0729842931937</v>
       </c>
@@ -8184,7 +8186,7 @@
         <f>IFERROR(IF('Datos'!$O13="","",'Datos'!$O13),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K13" s="13">
+      <c r="K13" s="23">
         <f>IFERROR(IF(OR($H13="",$I13="",$J13="",$D$33+$D$34+$J13&gt;=1),"",(1-$J13)*$H13*$I13*(1-($D$33+$D$34+$J13))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8192,7 +8194,7 @@
         <f>IFERROR(IF(OR($G13="",$K13=""),"",IF($G13&gt;=$K13,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="23">
         <f>IFERROR(IF(OR($G13="",$K13=""),"",$G13-$K13),"")</f>
         <v>-114.9614138215868</v>
       </c>
@@ -8225,7 +8227,7 @@
         <f>IFERROR(IF('Datos'!$F14="","",'Datos'!$F14),"")</f>
         <v>13.6</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="22">
         <f>IFERROR(IF(OR($D14="",$E14="",$F14="",$D$33+$D$34+$E14&gt;=1),"",(1-$E14)*$D14*$F14*(1-($D$33+$D$34+$E14))),"")</f>
         <v>1128.6370588235293</v>
       </c>
@@ -8241,7 +8243,7 @@
         <f>IFERROR(IF('Datos'!$O14="","",'Datos'!$O14),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="23">
         <f>IFERROR(IF(OR($H14="",$I14="",$J14="",$D$33+$D$34+$J14&gt;=1),"",(1-$J14)*$H14*$I14*(1-($D$33+$D$34+$J14))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8249,7 +8251,7 @@
         <f>IFERROR(IF(OR($G14="",$K14=""),"",IF($G14&gt;=$K14,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M14" s="13">
+      <c r="M14" s="23">
         <f>IFERROR(IF(OR($G14="",$K14=""),"",$G14-$K14),"")</f>
         <v>585.6026607087488</v>
       </c>
@@ -8282,7 +8284,7 @@
         <f>IFERROR(IF('Datos'!$F15="","",'Datos'!$F15),"")</f>
         <v>16.4</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="22">
         <f>IFERROR(IF(OR($D15="",$E15="",$F15="",$D$33+$D$34+$E15&gt;=1),"",(1-$E15)*$D15*$F15*(1-($D$33+$D$34+$E15))),"")</f>
         <v>556.1736585365852</v>
       </c>
@@ -8298,7 +8300,7 @@
         <f>IFERROR(IF('Datos'!$O15="","",'Datos'!$O15),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="23">
         <f>IFERROR(IF(OR($H15="",$I15="",$J15="",$D$33+$D$34+$J15&gt;=1),"",(1-$J15)*$H15*$I15*(1-($D$33+$D$34+$J15))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8306,7 +8308,7 @@
         <f>IFERROR(IF(OR($G15="",$K15=""),"",IF($G15&gt;=$K15,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M15" s="13">
+      <c r="M15" s="23">
         <f>IFERROR(IF(OR($G15="",$K15=""),"",$G15-$K15),"")</f>
         <v>13.139260421804693</v>
       </c>
@@ -8339,7 +8341,7 @@
         <f>IFERROR(IF('Datos'!$F16="","",'Datos'!$F16),"")</f>
         <v>32.7</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="22">
         <f>IFERROR(IF(OR($D16="",$E16="",$F16="",$D$33+$D$34+$E16&gt;=1),"",(1-$E16)*$D16*$F16*(1-($D$33+$D$34+$E16))),"")</f>
         <v>250.85180428134555</v>
       </c>
@@ -8355,7 +8357,7 @@
         <f>IFERROR(IF('Datos'!$O16="","",'Datos'!$O16),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K16" s="13">
+      <c r="K16" s="23">
         <f>IFERROR(IF(OR($H16="",$I16="",$J16="",$D$33+$D$34+$J16&gt;=1),"",(1-$J16)*$H16*$I16*(1-($D$33+$D$34+$J16))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8363,7 +8365,7 @@
         <f>IFERROR(IF(OR($G16="",$K16=""),"",IF($G16&gt;=$K16,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M16" s="13">
+      <c r="M16" s="23">
         <f>IFERROR(IF(OR($G16="",$K16=""),"",$G16-$K16),"")</f>
         <v>-292.18259383343496</v>
       </c>
@@ -8396,7 +8398,7 @@
         <f>IFERROR(IF('Datos'!$F17="","",'Datos'!$F17),"")</f>
         <v>21.8</v>
       </c>
-      <c r="G17" s="11">
+      <c r="G17" s="22">
         <f>IFERROR(IF(OR($D17="",$E17="",$F17="",$D$33+$D$34+$E17&gt;=1),"",(1-$E17)*$D17*$F17*(1-($D$33+$D$34+$E17))),"")</f>
         <v>177.23889908256876</v>
       </c>
@@ -8412,7 +8414,7 @@
         <f>IFERROR(IF('Datos'!$O17="","",'Datos'!$O17),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K17" s="13">
+      <c r="K17" s="23">
         <f>IFERROR(IF(OR($H17="",$I17="",$J17="",$D$33+$D$34+$J17&gt;=1),"",(1-$J17)*$H17*$I17*(1-($D$33+$D$34+$J17))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8420,7 +8422,7 @@
         <f>IFERROR(IF(OR($G17="",$K17=""),"",IF($G17&gt;=$K17,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M17" s="13">
+      <c r="M17" s="23">
         <f>IFERROR(IF(OR($G17="",$K17=""),"",$G17-$K17),"")</f>
         <v>-365.79549903221175</v>
       </c>
@@ -8453,7 +8455,7 @@
         <f>IFERROR(IF('Datos'!$F18="","",'Datos'!$F18),"")</f>
         <v>12.7</v>
       </c>
-      <c r="G18" s="11">
+      <c r="G18" s="22">
         <f>IFERROR(IF(OR($D18="",$E18="",$F18="",$D$33+$D$34+$E18&gt;=1),"",(1-$E18)*$D18*$F18*(1-($D$33+$D$34+$E18))),"")</f>
         <v>779.3858267716532</v>
       </c>
@@ -8469,7 +8471,7 @@
         <f>IFERROR(IF('Datos'!$O18="","",'Datos'!$O18),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K18" s="13">
+      <c r="K18" s="23">
         <f>IFERROR(IF(OR($H18="",$I18="",$J18="",$D$33+$D$34+$J18&gt;=1),"",(1-$J18)*$H18*$I18*(1-($D$33+$D$34+$J18))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8477,7 +8479,7 @@
         <f>IFERROR(IF(OR($G18="",$K18=""),"",IF($G18&gt;=$K18,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M18" s="13">
+      <c r="M18" s="23">
         <f>IFERROR(IF(OR($G18="",$K18=""),"",$G18-$K18),"")</f>
         <v>236.3514286568727</v>
       </c>
@@ -8510,7 +8512,7 @@
         <f>IFERROR(IF('Datos'!$F19="","",'Datos'!$F19),"")</f>
         <v>11.4</v>
       </c>
-      <c r="G19" s="11">
+      <c r="G19" s="22">
         <f>IFERROR(IF(OR($D19="",$E19="",$F19="",$D$33+$D$34+$E19&gt;=1),"",(1-$E19)*$D19*$F19*(1-($D$33+$D$34+$E19))),"")</f>
         <v>433.57754385964915</v>
       </c>
@@ -8526,7 +8528,7 @@
         <f>IFERROR(IF('Datos'!$O19="","",'Datos'!$O19),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K19" s="13">
+      <c r="K19" s="23">
         <f>IFERROR(IF(OR($H19="",$I19="",$J19="",$D$33+$D$34+$J19&gt;=1),"",(1-$J19)*$H19*$I19*(1-($D$33+$D$34+$J19))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8534,7 +8536,7 @@
         <f>IFERROR(IF(OR($G19="",$K19=""),"",IF($G19&gt;=$K19,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M19" s="13">
+      <c r="M19" s="23">
         <f>IFERROR(IF(OR($G19="",$K19=""),"",$G19-$K19),"")</f>
         <v>-109.45685425513136</v>
       </c>
@@ -8567,7 +8569,7 @@
         <f>IFERROR(IF('Datos'!$F20="","",'Datos'!$F20),"")</f>
         <v>22.4</v>
       </c>
-      <c r="G20" s="11">
+      <c r="G20" s="22">
         <f>IFERROR(IF(OR($D20="",$E20="",$F20="",$D$33+$D$34+$E20&gt;=1),"",(1-$E20)*$D20*$F20*(1-($D$33+$D$34+$E20))),"")</f>
         <v>251.9771428571427</v>
       </c>
@@ -8583,7 +8585,7 @@
         <f>IFERROR(IF('Datos'!$O20="","",'Datos'!$O20),"")</f>
         <v>0.3558752289242039</v>
       </c>
-      <c r="K20" s="13">
+      <c r="K20" s="23">
         <f>IFERROR(IF(OR($H20="",$I20="",$J20="",$D$33+$D$34+$J20&gt;=1),"",(1-$J20)*$H20*$I20*(1-($D$33+$D$34+$J20))),"")</f>
         <v>543.0343981147805</v>
       </c>
@@ -8591,7 +8593,7 @@
         <f>IFERROR(IF(OR($G20="",$K20=""),"",IF($G20&gt;=$K20,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M20" s="13">
+      <c r="M20" s="23">
         <f>IFERROR(IF(OR($G20="",$K20=""),"",$G20-$K20),"")</f>
         <v>-291.05725525763785</v>
       </c>
@@ -8624,7 +8626,7 @@
         <f>IFERROR(IF('Datos'!$F21="","",'Datos'!$F21),"")</f>
         <v>5.9</v>
       </c>
-      <c r="G21" s="11">
+      <c r="G21" s="22">
         <f>IFERROR(IF(OR($D21="",$E21="",$F21="",$D$33+$D$34+$E21&gt;=1),"",(1-$E21)*$D21*$F21*(1-($D$33+$D$34+$E21))),"")</f>
         <v>860.309152542373</v>
       </c>
@@ -8640,7 +8642,7 @@
         <f>IFERROR(IF('Datos'!$O21="","",'Datos'!$O21),"")</f>
         <v>0.2322985165927512</v>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="23">
         <f>IFERROR(IF(OR($H21="",$I21="",$J21="",$D$33+$D$34+$J21&gt;=1),"",(1-$J21)*$H21*$I21*(1-($D$33+$D$34+$J21))),"")</f>
         <v>436.3653616760971</v>
       </c>
@@ -8648,7 +8650,7 @@
         <f>IFERROR(IF(OR($G21="",$K21=""),"",IF($G21&gt;=$K21,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M21" s="13">
+      <c r="M21" s="23">
         <f>IFERROR(IF(OR($G21="",$K21=""),"",$G21-$K21),"")</f>
         <v>423.9437908662759</v>
       </c>
@@ -8681,7 +8683,7 @@
         <f>IFERROR(IF('Datos'!$F22="","",'Datos'!$F22),"")</f>
         <v>5.5</v>
       </c>
-      <c r="G22" s="11">
+      <c r="G22" s="22">
         <f>IFERROR(IF(OR($D22="",$E22="",$F22="",$D$33+$D$34+$E22&gt;=1),"",(1-$E22)*$D22*$F22*(1-($D$33+$D$34+$E22))),"")</f>
         <v>351.1199999999999</v>
       </c>
@@ -8697,7 +8699,7 @@
         <f>IFERROR(IF('Datos'!$O22="","",'Datos'!$O22),"")</f>
         <v>0.2322985165927512</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="23">
         <f>IFERROR(IF(OR($H22="",$I22="",$J22="",$D$33+$D$34+$J22&gt;=1),"",(1-$J22)*$H22*$I22*(1-($D$33+$D$34+$J22))),"")</f>
         <v>436.3653616760971</v>
       </c>
@@ -8705,7 +8707,7 @@
         <f>IFERROR(IF(OR($G22="",$K22=""),"",IF($G22&gt;=$K22,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M22" s="13">
+      <c r="M22" s="23">
         <f>IFERROR(IF(OR($G22="",$K22=""),"",$G22-$K22),"")</f>
         <v>-85.24536167609722</v>
       </c>
@@ -8738,7 +8740,7 @@
         <f>IFERROR(IF('Datos'!$F23="","",'Datos'!$F23),"")</f>
         <v>6.2</v>
       </c>
-      <c r="G23" s="11">
+      <c r="G23" s="22">
         <f>IFERROR(IF(OR($D23="",$E23="",$F23="",$D$33+$D$34+$E23&gt;=1),"",(1-$E23)*$D23*$F23*(1-($D$33+$D$34+$E23))),"")</f>
         <v>488.69806451612897</v>
       </c>
@@ -8754,7 +8756,7 @@
         <f>IFERROR(IF('Datos'!$O23="","",'Datos'!$O23),"")</f>
         <v>0.2322985165927512</v>
       </c>
-      <c r="K23" s="13">
+      <c r="K23" s="23">
         <f>IFERROR(IF(OR($H23="",$I23="",$J23="",$D$33+$D$34+$J23&gt;=1),"",(1-$J23)*$H23*$I23*(1-($D$33+$D$34+$J23))),"")</f>
         <v>436.3653616760971</v>
       </c>
@@ -8762,7 +8764,7 @@
         <f>IFERROR(IF(OR($G23="",$K23=""),"",IF($G23&gt;=$K23,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="M23" s="13">
+      <c r="M23" s="23">
         <f>IFERROR(IF(OR($G23="",$K23=""),"",$G23-$K23),"")</f>
         <v>52.33270284003186</v>
       </c>
@@ -8795,7 +8797,7 @@
         <f>IFERROR(IF('Datos'!$F24="","",'Datos'!$F24),"")</f>
         <v>4.5</v>
       </c>
-      <c r="G24" s="11">
+      <c r="G24" s="22">
         <f>IFERROR(IF(OR($D24="",$E24="",$F24="",$D$33+$D$34+$E24&gt;=1),"",(1-$E24)*$D24*$F24*(1-($D$33+$D$34+$E24))),"")</f>
         <v>50.01333333333333</v>
       </c>
@@ -8811,7 +8813,7 @@
         <f>IFERROR(IF('Datos'!$O24="","",'Datos'!$O24),"")</f>
         <v>0.2322985165927512</v>
       </c>
-      <c r="K24" s="13">
+      <c r="K24" s="23">
         <f>IFERROR(IF(OR($H24="",$I24="",$J24="",$D$33+$D$34+$J24&gt;=1),"",(1-$J24)*$H24*$I24*(1-($D$33+$D$34+$J24))),"")</f>
         <v>436.3653616760971</v>
       </c>
@@ -8819,7 +8821,7 @@
         <f>IFERROR(IF(OR($G24="",$K24=""),"",IF($G24&gt;=$K24,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="M24" s="13">
+      <c r="M24" s="23">
         <f>IFERROR(IF(OR($G24="",$K24=""),"",$G24-$K24),"")</f>
         <v>-386.3520283427638</v>
       </c>
@@ -8852,7 +8854,7 @@
         <f>IFERROR(IF('Datos'!$F25="","",'Datos'!$F25),"")</f>
         <v/>
       </c>
-      <c r="G25" s="11">
+      <c r="G25" s="22">
         <f>IFERROR(IF(OR($D25="",$E25="",$F25="",$D$33+$D$34+$E25&gt;=1),"",(1-$E25)*$D25*$F25*(1-($D$33+$D$34+$E25))),"")</f>
         <v/>
       </c>
@@ -8868,7 +8870,7 @@
         <f>IFERROR(IF('Datos'!$O25="","",'Datos'!$O25),"")</f>
         <v/>
       </c>
-      <c r="K25" s="13">
+      <c r="K25" s="23">
         <f>IFERROR(IF(OR($H25="",$I25="",$J25="",$D$33+$D$34+$J25&gt;=1),"",(1-$J25)*$H25*$I25*(1-($D$33+$D$34+$J25))),"")</f>
         <v/>
       </c>
@@ -8876,7 +8878,7 @@
         <f>IFERROR(IF(OR($G25="",$K25=""),"",IF($G25&gt;=$K25,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v/>
       </c>
-      <c r="M25" s="13">
+      <c r="M25" s="23">
         <f>IFERROR(IF(OR($G25="",$K25=""),"",$G25-$K25),"")</f>
         <v/>
       </c>
@@ -8909,7 +8911,7 @@
         <f>IFERROR(IF('Datos'!$F26="","",'Datos'!$F26),"")</f>
         <v/>
       </c>
-      <c r="G26" s="11">
+      <c r="G26" s="22">
         <f>IFERROR(IF(OR($D26="",$E26="",$F26="",$D$33+$D$34+$E26&gt;=1),"",(1-$E26)*$D26*$F26*(1-($D$33+$D$34+$E26))),"")</f>
         <v/>
       </c>
@@ -8925,7 +8927,7 @@
         <f>IFERROR(IF('Datos'!$O26="","",'Datos'!$O26),"")</f>
         <v/>
       </c>
-      <c r="K26" s="13">
+      <c r="K26" s="23">
         <f>IFERROR(IF(OR($H26="",$I26="",$J26="",$D$33+$D$34+$J26&gt;=1),"",(1-$J26)*$H26*$I26*(1-($D$33+$D$34+$J26))),"")</f>
         <v/>
       </c>
@@ -8933,7 +8935,7 @@
         <f>IFERROR(IF(OR($G26="",$K26=""),"",IF($G26&gt;=$K26,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v/>
       </c>
-      <c r="M26" s="13">
+      <c r="M26" s="23">
         <f>IFERROR(IF(OR($G26="",$K26=""),"",$G26-$K26),"")</f>
         <v/>
       </c>
@@ -8966,7 +8968,7 @@
         <f>IFERROR(IF('Datos'!$F27="","",'Datos'!$F27),"")</f>
         <v/>
       </c>
-      <c r="G27" s="11">
+      <c r="G27" s="22">
         <f>IFERROR(IF(OR($D27="",$E27="",$F27="",$D$33+$D$34+$E27&gt;=1),"",(1-$E27)*$D27*$F27*(1-($D$33+$D$34+$E27))),"")</f>
         <v/>
       </c>
@@ -8982,7 +8984,7 @@
         <f>IFERROR(IF('Datos'!$O27="","",'Datos'!$O27),"")</f>
         <v/>
       </c>
-      <c r="K27" s="13">
+      <c r="K27" s="23">
         <f>IFERROR(IF(OR($H27="",$I27="",$J27="",$D$33+$D$34+$J27&gt;=1),"",(1-$J27)*$H27*$I27*(1-($D$33+$D$34+$J27))),"")</f>
         <v/>
       </c>
@@ -8990,7 +8992,7 @@
         <f>IFERROR(IF(OR($G27="",$K27=""),"",IF($G27&gt;=$K27,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v/>
       </c>
-      <c r="M27" s="13">
+      <c r="M27" s="23">
         <f>IFERROR(IF(OR($G27="",$K27=""),"",$G27-$K27),"")</f>
         <v/>
       </c>
@@ -9023,7 +9025,7 @@
         <f>IFERROR(IF('Datos'!$F28="","",'Datos'!$F28),"")</f>
         <v/>
       </c>
-      <c r="G28" s="11">
+      <c r="G28" s="22">
         <f>IFERROR(IF(OR($D28="",$E28="",$F28="",$D$33+$D$34+$E28&gt;=1),"",(1-$E28)*$D28*$F28*(1-($D$33+$D$34+$E28))),"")</f>
         <v/>
       </c>
@@ -9039,7 +9041,7 @@
         <f>IFERROR(IF('Datos'!$O28="","",'Datos'!$O28),"")</f>
         <v/>
       </c>
-      <c r="K28" s="13">
+      <c r="K28" s="23">
         <f>IFERROR(IF(OR($H28="",$I28="",$J28="",$D$33+$D$34+$J28&gt;=1),"",(1-$J28)*$H28*$I28*(1-($D$33+$D$34+$J28))),"")</f>
         <v/>
       </c>
@@ -9047,7 +9049,7 @@
         <f>IFERROR(IF(OR($G28="",$K28=""),"",IF($G28&gt;=$K28,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v/>
       </c>
-      <c r="M28" s="13">
+      <c r="M28" s="23">
         <f>IFERROR(IF(OR($G28="",$K28=""),"",$G28-$K28),"")</f>
         <v/>
       </c>
@@ -9080,7 +9082,7 @@
         <f>IFERROR(IF('Datos'!$F29="","",'Datos'!$F29),"")</f>
         <v/>
       </c>
-      <c r="G29" s="11">
+      <c r="G29" s="22">
         <f>IFERROR(IF(OR($D29="",$E29="",$F29="",$D$33+$D$34+$E29&gt;=1),"",(1-$E29)*$D29*$F29*(1-($D$33+$D$34+$E29))),"")</f>
         <v/>
       </c>
@@ -9096,7 +9098,7 @@
         <f>IFERROR(IF('Datos'!$O29="","",'Datos'!$O29),"")</f>
         <v/>
       </c>
-      <c r="K29" s="13">
+      <c r="K29" s="23">
         <f>IFERROR(IF(OR($H29="",$I29="",$J29="",$D$33+$D$34+$J29&gt;=1),"",(1-$J29)*$H29*$I29*(1-($D$33+$D$34+$J29))),"")</f>
         <v/>
       </c>
@@ -9104,7 +9106,7 @@
         <f>IFERROR(IF(OR($G29="",$K29=""),"",IF($G29&gt;=$K29,"Por encima del objetivo","Por debajo del objetivo")),"")</f>
         <v/>
       </c>
-      <c r="M29" s="13">
+      <c r="M29" s="23">
         <f>IFERROR(IF(OR($G29="",$K29=""),"",$G29-$K29),"")</f>
         <v/>
       </c>
@@ -9155,10 +9157,10 @@
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>Goal Value medio de la carta (€)</t>
-        </is>
-      </c>
-      <c r="D35" s="13">
+          <t>Goal Value medio de la carta (índice)</t>
+        </is>
+      </c>
+      <c r="D35" s="23">
         <f>IFERROR(AVERAGE($G$5:$G$29),"")</f>
         <v>520.5515932949959</v>
       </c>
@@ -9336,11 +9338,11 @@
         <f>IFERROR(IF('Goal Value'!$L5="","",'Goal Value'!$L5),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="24">
         <f>IFERROR(IF($B5="","",IF($D5="Star",0,1)+IF($E5="Winner",0,1)+IF($F5="Prime",0,1)+IF($G5="Por encima del objetivo",0,1)),"")</f>
         <v>1.0</v>
       </c>
-      <c r="I5" s="23" t="str">
+      <c r="I5" s="25" t="str">
         <f>IFERROR(IF($B5="","",IF($H5=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D5="Dog",$E5="Loser",$F5="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D5="Plowhorse",$E5="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D5="Plowhorse",$E5="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G5&gt;='Datos'!$N5,'Datos'!$H5&gt;'Datos'!$O5),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D5="Puzzle",$E5="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F5="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G5="Por debajo del objetivo",$D5="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D5="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Popular con margen bajo: subir precio o bajar coste.</v>
       </c>
@@ -9377,11 +9379,11 @@
         <f>IFERROR(IF('Goal Value'!$L6="","",'Goal Value'!$L6),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="24">
         <f>IFERROR(IF($B6="","",IF($D6="Star",0,1)+IF($E6="Winner",0,1)+IF($F6="Prime",0,1)+IF($G6="Por encima del objetivo",0,1)),"")</f>
         <v>0.0</v>
       </c>
-      <c r="I6" s="23" t="str">
+      <c r="I6" s="25" t="str">
         <f>IFERROR(IF($B6="","",IF($H6=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D6="Dog",$E6="Loser",$F6="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D6="Plowhorse",$E6="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D6="Plowhorse",$E6="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G6&gt;='Datos'!$N6,'Datos'!$H6&gt;'Datos'!$O6),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D6="Puzzle",$E6="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F6="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G6="Por debajo del objetivo",$D6="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D6="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.</v>
       </c>
@@ -9418,11 +9420,11 @@
         <f>IFERROR(IF('Goal Value'!$L7="","",'Goal Value'!$L7),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="24">
         <f>IFERROR(IF($B7="","",IF($D7="Star",0,1)+IF($E7="Winner",0,1)+IF($F7="Prime",0,1)+IF($G7="Por encima del objetivo",0,1)),"")</f>
         <v>3.0</v>
       </c>
-      <c r="I7" s="23" t="str">
+      <c r="I7" s="25" t="str">
         <f>IFERROR(IF($B7="","",IF($H7=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D7="Dog",$E7="Loser",$F7="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D7="Plowhorse",$E7="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D7="Plowhorse",$E7="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G7&gt;='Datos'!$N7,'Datos'!$H7&gt;'Datos'!$O7),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D7="Puzzle",$E7="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F7="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G7="Por debajo del objetivo",$D7="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D7="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -9459,11 +9461,11 @@
         <f>IFERROR(IF('Goal Value'!$L8="","",'Goal Value'!$L8),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="24">
         <f>IFERROR(IF($B8="","",IF($D8="Star",0,1)+IF($E8="Winner",0,1)+IF($F8="Prime",0,1)+IF($G8="Por encima del objetivo",0,1)),"")</f>
         <v>1.0</v>
       </c>
-      <c r="I8" s="23" t="str">
+      <c r="I8" s="25" t="str">
         <f>IFERROR(IF($B8="","",IF($H8=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D8="Dog",$E8="Loser",$F8="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D8="Plowhorse",$E8="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D8="Plowhorse",$E8="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G8&gt;='Datos'!$N8,'Datos'!$H8&gt;'Datos'!$O8),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D8="Puzzle",$E8="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F8="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G8="Por debajo del objetivo",$D8="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D8="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Popular con margen bajo: subir precio o bajar coste.</v>
       </c>
@@ -9500,11 +9502,11 @@
         <f>IFERROR(IF('Goal Value'!$L9="","",'Goal Value'!$L9),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="24">
         <f>IFERROR(IF($B9="","",IF($D9="Star",0,1)+IF($E9="Winner",0,1)+IF($F9="Prime",0,1)+IF($G9="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I9" s="23" t="str">
+      <c r="I9" s="25" t="str">
         <f>IFERROR(IF($B9="","",IF($H9=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D9="Dog",$E9="Loser",$F9="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D9="Plowhorse",$E9="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D9="Plowhorse",$E9="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G9&gt;='Datos'!$N9,'Datos'!$H9&gt;'Datos'!$O9),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D9="Puzzle",$E9="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F9="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G9="Por debajo del objetivo",$D9="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D9="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -9541,11 +9543,11 @@
         <f>IFERROR(IF('Goal Value'!$L10="","",'Goal Value'!$L10),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="24">
         <f>IFERROR(IF($B10="","",IF($D10="Star",0,1)+IF($E10="Winner",0,1)+IF($F10="Prime",0,1)+IF($G10="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I10" s="23" t="str">
+      <c r="I10" s="25" t="str">
         <f>IFERROR(IF($B10="","",IF($H10=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D10="Dog",$E10="Loser",$F10="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D10="Plowhorse",$E10="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D10="Plowhorse",$E10="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G10&gt;='Datos'!$N10,'Datos'!$H10&gt;'Datos'!$O10),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D10="Puzzle",$E10="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F10="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G10="Por debajo del objetivo",$D10="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D10="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.</v>
       </c>
@@ -9582,11 +9584,11 @@
         <f>IFERROR(IF('Goal Value'!$L11="","",'Goal Value'!$L11),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="24">
         <f>IFERROR(IF($B11="","",IF($D11="Star",0,1)+IF($E11="Winner",0,1)+IF($F11="Prime",0,1)+IF($G11="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I11" s="23" t="str">
+      <c r="I11" s="25" t="str">
         <f>IFERROR(IF($B11="","",IF($H11=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D11="Dog",$E11="Loser",$F11="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D11="Plowhorse",$E11="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D11="Plowhorse",$E11="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G11&gt;='Datos'!$N11,'Datos'!$H11&gt;'Datos'!$O11),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D11="Puzzle",$E11="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F11="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G11="Por debajo del objetivo",$D11="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D11="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.</v>
       </c>
@@ -9623,11 +9625,11 @@
         <f>IFERROR(IF('Goal Value'!$L12="","",'Goal Value'!$L12),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="24">
         <f>IFERROR(IF($B12="","",IF($D12="Star",0,1)+IF($E12="Winner",0,1)+IF($F12="Prime",0,1)+IF($G12="Por encima del objetivo",0,1)),"")</f>
         <v>0.0</v>
       </c>
-      <c r="I12" s="23" t="str">
+      <c r="I12" s="25" t="str">
         <f>IFERROR(IF($B12="","",IF($H12=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D12="Dog",$E12="Loser",$F12="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D12="Plowhorse",$E12="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D12="Plowhorse",$E12="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G12&gt;='Datos'!$N12,'Datos'!$H12&gt;'Datos'!$O12),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D12="Puzzle",$E12="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F12="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G12="Por debajo del objetivo",$D12="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D12="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.</v>
       </c>
@@ -9664,11 +9666,11 @@
         <f>IFERROR(IF('Goal Value'!$L13="","",'Goal Value'!$L13),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="24">
         <f>IFERROR(IF($B13="","",IF($D13="Star",0,1)+IF($E13="Winner",0,1)+IF($F13="Prime",0,1)+IF($G13="Por encima del objetivo",0,1)),"")</f>
         <v>3.0</v>
       </c>
-      <c r="I13" s="23" t="str">
+      <c r="I13" s="25" t="str">
         <f>IFERROR(IF($B13="","",IF($H13=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D13="Dog",$E13="Loser",$F13="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D13="Plowhorse",$E13="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D13="Plowhorse",$E13="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G13&gt;='Datos'!$N13,'Datos'!$H13&gt;'Datos'!$O13),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D13="Puzzle",$E13="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F13="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G13="Por debajo del objetivo",$D13="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D13="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -9705,11 +9707,11 @@
         <f>IFERROR(IF('Goal Value'!$L14="","",'Goal Value'!$L14),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="24">
         <f>IFERROR(IF($B14="","",IF($D14="Star",0,1)+IF($E14="Winner",0,1)+IF($F14="Prime",0,1)+IF($G14="Por encima del objetivo",0,1)),"")</f>
         <v>1.0</v>
       </c>
-      <c r="I14" s="23" t="str">
+      <c r="I14" s="25" t="str">
         <f>IFERROR(IF($B14="","",IF($H14=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D14="Dog",$E14="Loser",$F14="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D14="Plowhorse",$E14="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D14="Plowhorse",$E14="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G14&gt;='Datos'!$N14,'Datos'!$H14&gt;'Datos'!$O14),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D14="Puzzle",$E14="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F14="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G14="Por debajo del objetivo",$D14="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D14="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Popular con margen bajo: subir precio o bajar coste.</v>
       </c>
@@ -9746,11 +9748,11 @@
         <f>IFERROR(IF('Goal Value'!$L15="","",'Goal Value'!$L15),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="24">
         <f>IFERROR(IF($B15="","",IF($D15="Star",0,1)+IF($E15="Winner",0,1)+IF($F15="Prime",0,1)+IF($G15="Por encima del objetivo",0,1)),"")</f>
         <v>3.0</v>
       </c>
-      <c r="I15" s="23" t="str">
+      <c r="I15" s="25" t="str">
         <f>IFERROR(IF($B15="","",IF($H15=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D15="Dog",$E15="Loser",$F15="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D15="Plowhorse",$E15="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D15="Plowhorse",$E15="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G15&gt;='Datos'!$N15,'Datos'!$H15&gt;'Datos'!$O15),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D15="Puzzle",$E15="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F15="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G15="Por debajo del objetivo",$D15="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D15="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.</v>
       </c>
@@ -9787,11 +9789,11 @@
         <f>IFERROR(IF('Goal Value'!$L16="","",'Goal Value'!$L16),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="24">
         <f>IFERROR(IF($B16="","",IF($D16="Star",0,1)+IF($E16="Winner",0,1)+IF($F16="Prime",0,1)+IF($G16="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I16" s="23" t="str">
+      <c r="I16" s="25" t="str">
         <f>IFERROR(IF($B16="","",IF($H16=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D16="Dog",$E16="Loser",$F16="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D16="Plowhorse",$E16="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D16="Plowhorse",$E16="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G16&gt;='Datos'!$N16,'Datos'!$H16&gt;'Datos'!$O16),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D16="Puzzle",$E16="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F16="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G16="Por debajo del objetivo",$D16="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D16="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -9828,11 +9830,11 @@
         <f>IFERROR(IF('Goal Value'!$L17="","",'Goal Value'!$L17),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H17" s="22">
+      <c r="H17" s="24">
         <f>IFERROR(IF($B17="","",IF($D17="Star",0,1)+IF($E17="Winner",0,1)+IF($F17="Prime",0,1)+IF($G17="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I17" s="23" t="str">
+      <c r="I17" s="25" t="str">
         <f>IFERROR(IF($B17="","",IF($H17=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D17="Dog",$E17="Loser",$F17="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D17="Plowhorse",$E17="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D17="Plowhorse",$E17="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G17&gt;='Datos'!$N17,'Datos'!$H17&gt;'Datos'!$O17),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D17="Puzzle",$E17="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F17="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G17="Por debajo del objetivo",$D17="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D17="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -9869,11 +9871,11 @@
         <f>IFERROR(IF('Goal Value'!$L18="","",'Goal Value'!$L18),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H18" s="22">
+      <c r="H18" s="24">
         <f>IFERROR(IF($B18="","",IF($D18="Star",0,1)+IF($E18="Winner",0,1)+IF($F18="Prime",0,1)+IF($G18="Por encima del objetivo",0,1)),"")</f>
         <v>1.0</v>
       </c>
-      <c r="I18" s="23" t="str">
+      <c r="I18" s="25" t="str">
         <f>IFERROR(IF($B18="","",IF($H18=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D18="Dog",$E18="Loser",$F18="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D18="Plowhorse",$E18="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D18="Plowhorse",$E18="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G18&gt;='Datos'!$N18,'Datos'!$H18&gt;'Datos'!$O18),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D18="Puzzle",$E18="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F18="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G18="Por debajo del objetivo",$D18="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D18="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Popular con margen bajo: subir precio o bajar coste.</v>
       </c>
@@ -9910,11 +9912,11 @@
         <f>IFERROR(IF('Goal Value'!$L19="","",'Goal Value'!$L19),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="24">
         <f>IFERROR(IF($B19="","",IF($D19="Star",0,1)+IF($E19="Winner",0,1)+IF($F19="Prime",0,1)+IF($G19="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I19" s="23" t="str">
+      <c r="I19" s="25" t="str">
         <f>IFERROR(IF($B19="","",IF($H19=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D19="Dog",$E19="Loser",$F19="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D19="Plowhorse",$E19="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D19="Plowhorse",$E19="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G19&gt;='Datos'!$N19,'Datos'!$H19&gt;'Datos'!$O19),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D19="Puzzle",$E19="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F19="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G19="Por debajo del objetivo",$D19="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D19="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.</v>
       </c>
@@ -9951,11 +9953,11 @@
         <f>IFERROR(IF('Goal Value'!$L20="","",'Goal Value'!$L20),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="24">
         <f>IFERROR(IF($B20="","",IF($D20="Star",0,1)+IF($E20="Winner",0,1)+IF($F20="Prime",0,1)+IF($G20="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I20" s="23" t="str">
+      <c r="I20" s="25" t="str">
         <f>IFERROR(IF($B20="","",IF($H20=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D20="Dog",$E20="Loser",$F20="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D20="Plowhorse",$E20="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D20="Plowhorse",$E20="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G20&gt;='Datos'!$N20,'Datos'!$H20&gt;'Datos'!$O20),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D20="Puzzle",$E20="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F20="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G20="Por debajo del objetivo",$D20="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D20="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -9992,11 +9994,11 @@
         <f>IFERROR(IF('Goal Value'!$L21="","",'Goal Value'!$L21),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H21" s="22">
+      <c r="H21" s="24">
         <f>IFERROR(IF($B21="","",IF($D21="Star",0,1)+IF($E21="Winner",0,1)+IF($F21="Prime",0,1)+IF($G21="Por encima del objetivo",0,1)),"")</f>
         <v>0.0</v>
       </c>
-      <c r="I21" s="23" t="str">
+      <c r="I21" s="25" t="str">
         <f>IFERROR(IF($B21="","",IF($H21=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D21="Dog",$E21="Loser",$F21="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D21="Plowhorse",$E21="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D21="Plowhorse",$E21="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G21&gt;='Datos'!$N21,'Datos'!$H21&gt;'Datos'!$O21),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D21="Puzzle",$E21="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F21="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G21="Por debajo del objetivo",$D21="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D21="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.</v>
       </c>
@@ -10033,11 +10035,11 @@
         <f>IFERROR(IF('Goal Value'!$L22="","",'Goal Value'!$L22),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="24">
         <f>IFERROR(IF($B22="","",IF($D22="Star",0,1)+IF($E22="Winner",0,1)+IF($F22="Prime",0,1)+IF($G22="Por encima del objetivo",0,1)),"")</f>
         <v>3.0</v>
       </c>
-      <c r="I22" s="23" t="str">
+      <c r="I22" s="25" t="str">
         <f>IFERROR(IF($B22="","",IF($H22=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D22="Dog",$E22="Loser",$F22="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D22="Plowhorse",$E22="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D22="Plowhorse",$E22="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G22&gt;='Datos'!$N22,'Datos'!$H22&gt;'Datos'!$O22),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D22="Puzzle",$E22="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F22="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G22="Por debajo del objetivo",$D22="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D22="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Popular con margen bajo: subir precio o bajar coste.</v>
       </c>
@@ -10074,11 +10076,11 @@
         <f>IFERROR(IF('Goal Value'!$L23="","",'Goal Value'!$L23),"")</f>
         <v>Por encima del objetivo</v>
       </c>
-      <c r="H23" s="22">
+      <c r="H23" s="24">
         <f>IFERROR(IF($B23="","",IF($D23="Star",0,1)+IF($E23="Winner",0,1)+IF($F23="Prime",0,1)+IF($G23="Por encima del objetivo",0,1)),"")</f>
         <v>2.0</v>
       </c>
-      <c r="I23" s="23" t="str">
+      <c r="I23" s="25" t="str">
         <f>IFERROR(IF($B23="","",IF($H23=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D23="Dog",$E23="Loser",$F23="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D23="Plowhorse",$E23="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D23="Plowhorse",$E23="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G23&gt;='Datos'!$N23,'Datos'!$H23&gt;'Datos'!$O23),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D23="Puzzle",$E23="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F23="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G23="Por debajo del objetivo",$D23="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D23="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.</v>
       </c>
@@ -10115,11 +10117,11 @@
         <f>IFERROR(IF('Goal Value'!$L24="","",'Goal Value'!$L24),"")</f>
         <v>Por debajo del objetivo</v>
       </c>
-      <c r="H24" s="22">
+      <c r="H24" s="24">
         <f>IFERROR(IF($B24="","",IF($D24="Star",0,1)+IF($E24="Winner",0,1)+IF($F24="Prime",0,1)+IF($G24="Por encima del objetivo",0,1)),"")</f>
         <v>4.0</v>
       </c>
-      <c r="I24" s="23" t="str">
+      <c r="I24" s="25" t="str">
         <f>IFERROR(IF($B24="","",IF($H24=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D24="Dog",$E24="Loser",$F24="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D24="Plowhorse",$E24="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D24="Plowhorse",$E24="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G24&gt;='Datos'!$N24,'Datos'!$H24&gt;'Datos'!$O24),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D24="Puzzle",$E24="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F24="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G24="Por debajo del objetivo",$D24="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D24="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v>Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.</v>
       </c>
@@ -10156,11 +10158,11 @@
         <f>IFERROR(IF('Goal Value'!$L25="","",'Goal Value'!$L25),"")</f>
         <v/>
       </c>
-      <c r="H25" s="22">
+      <c r="H25" s="24">
         <f>IFERROR(IF($B25="","",IF($D25="Star",0,1)+IF($E25="Winner",0,1)+IF($F25="Prime",0,1)+IF($G25="Por encima del objetivo",0,1)),"")</f>
         <v/>
       </c>
-      <c r="I25" s="23">
+      <c r="I25" s="25">
         <f>IFERROR(IF($B25="","",IF($H25=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D25="Dog",$E25="Loser",$F25="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D25="Plowhorse",$E25="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D25="Plowhorse",$E25="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G25&gt;='Datos'!$N25,'Datos'!$H25&gt;'Datos'!$O25),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D25="Puzzle",$E25="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F25="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G25="Por debajo del objetivo",$D25="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D25="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v/>
       </c>
@@ -10197,11 +10199,11 @@
         <f>IFERROR(IF('Goal Value'!$L26="","",'Goal Value'!$L26),"")</f>
         <v/>
       </c>
-      <c r="H26" s="22">
+      <c r="H26" s="24">
         <f>IFERROR(IF($B26="","",IF($D26="Star",0,1)+IF($E26="Winner",0,1)+IF($F26="Prime",0,1)+IF($G26="Por encima del objetivo",0,1)),"")</f>
         <v/>
       </c>
-      <c r="I26" s="23">
+      <c r="I26" s="25">
         <f>IFERROR(IF($B26="","",IF($H26=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D26="Dog",$E26="Loser",$F26="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D26="Plowhorse",$E26="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D26="Plowhorse",$E26="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G26&gt;='Datos'!$N26,'Datos'!$H26&gt;'Datos'!$O26),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D26="Puzzle",$E26="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F26="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G26="Por debajo del objetivo",$D26="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D26="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v/>
       </c>
@@ -10238,11 +10240,11 @@
         <f>IFERROR(IF('Goal Value'!$L27="","",'Goal Value'!$L27),"")</f>
         <v/>
       </c>
-      <c r="H27" s="22">
+      <c r="H27" s="24">
         <f>IFERROR(IF($B27="","",IF($D27="Star",0,1)+IF($E27="Winner",0,1)+IF($F27="Prime",0,1)+IF($G27="Por encima del objetivo",0,1)),"")</f>
         <v/>
       </c>
-      <c r="I27" s="23">
+      <c r="I27" s="25">
         <f>IFERROR(IF($B27="","",IF($H27=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D27="Dog",$E27="Loser",$F27="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D27="Plowhorse",$E27="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D27="Plowhorse",$E27="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G27&gt;='Datos'!$N27,'Datos'!$H27&gt;'Datos'!$O27),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D27="Puzzle",$E27="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F27="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G27="Por debajo del objetivo",$D27="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D27="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v/>
       </c>
@@ -10279,11 +10281,11 @@
         <f>IFERROR(IF('Goal Value'!$L28="","",'Goal Value'!$L28),"")</f>
         <v/>
       </c>
-      <c r="H28" s="22">
+      <c r="H28" s="24">
         <f>IFERROR(IF($B28="","",IF($D28="Star",0,1)+IF($E28="Winner",0,1)+IF($F28="Prime",0,1)+IF($G28="Por encima del objetivo",0,1)),"")</f>
         <v/>
       </c>
-      <c r="I28" s="23">
+      <c r="I28" s="25">
         <f>IFERROR(IF($B28="","",IF($H28=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D28="Dog",$E28="Loser",$F28="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D28="Plowhorse",$E28="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D28="Plowhorse",$E28="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G28&gt;='Datos'!$N28,'Datos'!$H28&gt;'Datos'!$O28),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D28="Puzzle",$E28="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F28="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G28="Por debajo del objetivo",$D28="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D28="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v/>
       </c>
@@ -10320,11 +10322,11 @@
         <f>IFERROR(IF('Goal Value'!$L29="","",'Goal Value'!$L29),"")</f>
         <v/>
       </c>
-      <c r="H29" s="22">
+      <c r="H29" s="24">
         <f>IFERROR(IF($B29="","",IF($D29="Star",0,1)+IF($E29="Winner",0,1)+IF($F29="Prime",0,1)+IF($G29="Por encima del objetivo",0,1)),"")</f>
         <v/>
       </c>
-      <c r="I29" s="23">
+      <c r="I29" s="25">
         <f>IFERROR(IF($B29="","",IF($H29=0,"Las cuatro lecturas coinciden en lo mejor: mantener, destacar en carta y proteger receta y proveedor.",IF(AND($D29="Dog",$E29="Loser",$F29="Problem"),"Poco pedido, food cost alto y aporta poco margen al total: candidato a retirar o a reformular de raíz.",IF(AND($D29="Plowhorse",$E29="Winner"),"Popular con margen bajo: subir precio o bajar coste.",IF(AND($D29="Plowhorse",$E29="Loser"),"Popular pero caro de producir y de margen corto: reformular la receta antes de tocar el precio.",IF(AND('Datos'!$G29&gt;='Datos'!$N29,'Datos'!$H29&gt;'Datos'!$O29),"MC alto con food cost pobre: proteger el margen en euros, revisar precio, no retirar.",IF(AND($D29="Puzzle",$E29="Winner"),"Rentable y con food cost sano, pero poco pedido: es problema de carta, no de cocina. Renómbralo, súbelo de posición o que lo sugiera la sala.",IF($F29="Sleeper","Food cost sano pero aporta poco margen al total: dale visibilidad antes de retirarlo.",IF(AND($G29="Por debajo del objetivo",$D29="Star"),"Vende y deja margen, pero se queda por debajo del Goal Value de su familia: va justo de recorrido, revisa el precio.",IF($D29="Dog","Poco pedido: antes de retirarlo comprueba si es de temporada o si acompaña a otro plato que sí vende.","Las lecturas discrepan: cada método mide dos de las tres variables (popularidad, margen en euros y food cost). Decide con la que más te duela este mes.")))))))))),"")</f>
         <v/>
       </c>
@@ -10359,7 +10361,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="24" t="n">
+      <c r="B33" s="26" t="n">
         <v>0</v>
       </c>
       <c r="C33" s="8">
@@ -10372,7 +10374,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="24" t="n">
+      <c r="B34" s="26" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="8">
@@ -10385,7 +10387,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="24" t="n">
+      <c r="B35" s="26" t="n">
         <v>2</v>
       </c>
       <c r="C35" s="8">
@@ -10398,7 +10400,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="24" t="n">
+      <c r="B36" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C36" s="8">
@@ -10411,7 +10413,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="24" t="n">
+      <c r="B37" s="26" t="n">
         <v>4</v>
       </c>
       <c r="C37" s="8">
@@ -10835,7 +10837,7 @@
           <t>PVP del menú, sin IVA (€)</t>
         </is>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="27">
         <f>IFERROR(IF(OR($C$19="",$C$20=""),"",$C$19/(1+$C$20)),"")</f>
         <v>13.18181818181818</v>
       </c>
@@ -10935,7 +10937,7 @@
           <t>Primeros</t>
         </is>
       </c>
-      <c r="B27" s="26">
+      <c r="B27" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A27,$D$5:$D$16),"")</f>
         <v>1.0</v>
       </c>
@@ -10943,7 +10945,7 @@
         <f>IFERROR(SUMPRODUCT(--($A$5:$A$16=$A27),$C$5:$C$16,$D$5:$D$16),"")</f>
         <v>1.2625000000000002</v>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A27,$E$5:$E$16),"")</f>
         <v>1.0</v>
       </c>
@@ -10951,7 +10953,7 @@
         <f>IFERROR(SUMPRODUCT(--($A$5:$A$16=$A27),$C$5:$C$16,$E$5:$E$16),"")</f>
         <v>1.3650000000000002</v>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A27,$F$5:$F$16),"")</f>
         <v>1.0</v>
       </c>
@@ -10966,7 +10968,7 @@
           <t>Segundos</t>
         </is>
       </c>
-      <c r="B28" s="26">
+      <c r="B28" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A28,$D$5:$D$16),"")</f>
         <v>1.0</v>
       </c>
@@ -10974,7 +10976,7 @@
         <f>IFERROR(SUMPRODUCT(--($A$5:$A$16=$A28),$C$5:$C$16,$D$5:$D$16),"")</f>
         <v>3.2299999999999995</v>
       </c>
-      <c r="D28" s="26">
+      <c r="D28" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A28,$E$5:$E$16),"")</f>
         <v>1.0</v>
       </c>
@@ -10982,7 +10984,7 @@
         <f>IFERROR(SUMPRODUCT(--($A$5:$A$16=$A28),$C$5:$C$16,$E$5:$E$16),"")</f>
         <v>3.3949999999999996</v>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A28,$F$5:$F$16),"")</f>
         <v>1.0</v>
       </c>
@@ -10997,7 +10999,7 @@
           <t>Postres</t>
         </is>
       </c>
-      <c r="B29" s="26">
+      <c r="B29" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A29,$D$5:$D$16),"")</f>
         <v>1.0</v>
       </c>
@@ -11005,7 +11007,7 @@
         <f>IFERROR(SUMPRODUCT(--($A$5:$A$16=$A29),$C$5:$C$16,$D$5:$D$16),"")</f>
         <v>0.5900000000000001</v>
       </c>
-      <c r="D29" s="26">
+      <c r="D29" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A29,$E$5:$E$16),"")</f>
         <v>1.0</v>
       </c>
@@ -11013,7 +11015,7 @@
         <f>IFERROR(SUMPRODUCT(--($A$5:$A$16=$A29),$C$5:$C$16,$E$5:$E$16),"")</f>
         <v>0.62</v>
       </c>
-      <c r="F29" s="26">
+      <c r="F29" s="28">
         <f>IFERROR(SUMIF($A$5:$A$16,$A29,$F$5:$F$16),"")</f>
         <v>1.0</v>
       </c>
@@ -11160,15 +11162,15 @@
           <t>Food cost del menú (%)</t>
         </is>
       </c>
-      <c r="B39" s="27">
+      <c r="B39" s="29">
         <f>IFERROR(IF(OR($C$21="",$C$21=0,B38=""),"",B38/$C$21),"")</f>
         <v>0.42729310344827587</v>
       </c>
-      <c r="C39" s="27">
+      <c r="C39" s="29">
         <f>IFERROR(IF(OR($C$21="",$C$21=0,C38=""),"",C38/$C$21),"")</f>
         <v>0.4498620689655173</v>
       </c>
-      <c r="D39" s="27">
+      <c r="D39" s="29">
         <f>IFERROR(IF(OR($C$21="",$C$21=0,D38=""),"",D38/$C$21),"")</f>
         <v>0.406051724137931</v>
       </c>
@@ -11184,15 +11186,15 @@
           <t>Margen de contribución por menú (€)</t>
         </is>
       </c>
-      <c r="B40" s="25">
+      <c r="B40" s="27">
         <f>IFERROR(IF(OR($C$21="",B38=""),"",$C$21-B38),"")</f>
         <v>7.5493181818181805</v>
       </c>
-      <c r="C40" s="25">
+      <c r="C40" s="27">
         <f>IFERROR(IF(OR($C$21="",C38=""),"",$C$21-C38),"")</f>
         <v>7.25181818181818</v>
       </c>
-      <c r="D40" s="25">
+      <c r="D40" s="27">
         <f>IFERROR(IF(OR($C$21="",D38=""),"",$C$21-D38),"")</f>
         <v>7.829318181818181</v>
       </c>

</xml_diff>